<commit_message>
adiciona planilha dados e analise com as celulas devidamente preenchidas com analise dos poros
</commit_message>
<xml_diff>
--- a/planilhaModelo.xlsx
+++ b/planilhaModelo.xlsx
@@ -90,17 +90,17 @@
     <t>Incerteza Desvio Padrão</t>
   </si>
   <si>
-    <t>Variância</t>
-  </si>
-  <si>
-    <t>Coeficiente de variância</t>
+    <t>GERAL</t>
+  </si>
+  <si>
+    <t>Poro dominante</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,13 +112,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -147,7 +140,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -184,8 +177,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -212,12 +211,208 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="1"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -226,153 +421,170 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -669,41 +881,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="7" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
+      <c r="A3" s="25"/>
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
@@ -746,7 +958,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -761,119 +973,186 @@
     <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.28515625" customWidth="1"/>
+    <col min="13" max="13" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="3"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+    <row r="2" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="18" t="s">
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="39" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
+    <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="36"/>
+      <c r="B3" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="12" t="s">
         <v>13</v>
       </c>
+      <c r="M3" s="40"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="9"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="9"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
+      <c r="B6" s="9"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="9"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>20</v>
       </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="9"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="26"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="28"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B9" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:K1"/>
+  <mergeCells count="6">
+    <mergeCell ref="B8:M8"/>
     <mergeCell ref="C2:H2"/>
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="M2:M3"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>